<commit_message>
fix: align appearance table gender labels with enum
- Update appearance table gender values from MAN/WOMAN to MALE/FEMALE
</commit_message>
<xml_diff>
--- a/resources/table/appearance.xlsx
+++ b/resources/table/appearance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF89301-EFC7-4376-8660-1848FCF27350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4D1C73-F7D7-4110-BBDD-DB52103EBAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
@@ -75,10 +75,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MAN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>NORMAL</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -107,10 +103,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>WOMAN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>GHOST</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -123,6 +115,14 @@
   </si>
   <si>
     <t>gender</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MALE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FEMALE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -511,13 +511,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -535,7 +535,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>8</v>
@@ -549,31 +549,31 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>9</v>
@@ -625,7 +625,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
@@ -652,7 +652,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -660,7 +660,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
@@ -681,7 +681,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -689,7 +689,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
@@ -710,7 +710,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -718,7 +718,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C7" s="1">
         <v>0</v>
@@ -739,7 +739,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>